<commit_message>
Silviana ajusta datapackage, schema e arquivos de dados
</commit_message>
<xml_diff>
--- a/data/raw/projetos_acordo_judicial_reparacao_vale.xlsx
+++ b/data/raw/projetos_acordo_judicial_reparacao_vale.xlsx
@@ -1,25 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24931"/>
-  <workbookPr defaultThemeVersion="166925"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Silviana\Documents\1. CGE\tele-trabalho\GIT\transparencia-mg\acordo-judicial-reparacao-vale\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hugos\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F7E1FC1-9464-440E-88D6-79D32FCA3D5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20370" yWindow="-120" windowWidth="20730" windowHeight="11160" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="6750"/>
   </bookViews>
   <sheets>
-    <sheet name="projetos" sheetId="1" r:id="rId1"/>
+    <sheet name="projetos" sheetId="2" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">projetos!$D$1:$K$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">projetos!$D$1:$I$1</definedName>
   </definedNames>
-  <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <calcPr calcId="162913"/>
   <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
@@ -30,64 +32,220 @@
         <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
       </xcalcf:calcFeatures>
     </ext>
-    <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
-      <loext:extCalcPr stringRefSyntax="ExcelA1"/>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
-  <si>
-    <t>codigo_siafi</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="62">
+  <si>
+    <t>projeto</t>
   </si>
   <si>
     <t>anexo</t>
   </si>
   <si>
-    <t>codigo_orgao</t>
-  </si>
-  <si>
-    <t>orgao</t>
-  </si>
-  <si>
-    <t>projeto</t>
-  </si>
-  <si>
-    <t>valor_total_projeto</t>
+    <t>codigo_projeto</t>
+  </si>
+  <si>
+    <t>valor_projeto</t>
   </si>
   <si>
     <t>IV</t>
   </si>
   <si>
+    <t>II.3</t>
+  </si>
+  <si>
+    <t>III</t>
+  </si>
+  <si>
+    <t>Reestruturação logística, tecnológica e de cobrança da dívida ativa da AGE</t>
+  </si>
+  <si>
+    <t>Atualização do Plano Diretor de Desenvolvimento Integrado da Região Metropolitana de Belo Horizonte - PDDI-RMBH</t>
+  </si>
+  <si>
+    <t>Elaboração de Plano Metropolitano de Segurança Hídrica para a Região Metropolitana de Belo Horizonte.</t>
+  </si>
+  <si>
+    <t>Implantação do Sistema de Informações Regulatórias da ARSAE-MG</t>
+  </si>
+  <si>
+    <t>Execução de obras e serviços de engenharia em várias unidades do CBMMG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Expansão e fortalecimento da Academia do Corpo de Bombeiros Militar </t>
+  </si>
+  <si>
+    <t>Reestruturação das Tecnologias de Informação do CBMMG</t>
+  </si>
+  <si>
+    <t>Fortalecimento e reestruturação tecnológica da Controladoria Geral do Estado</t>
+  </si>
+  <si>
+    <t>Intervenções e Obras a serem realizadas, sob a responsabilidade e de propriedade do Estado de Minas Gerais, com o objetivo de aumentar a resiliência das Bacias do Paraopeba e Rio das Velhas, de modo a garantir o abastecimento da Região Metropolitana de Belo Horizonte - RMBH</t>
+  </si>
+  <si>
+    <t>Reestruturação dos Hospitais da Rede FHEMIG (Hospital Infantil João Paulo II, Hospital João XXIII e Hospital Júlia Kubitschek)</t>
+  </si>
+  <si>
+    <t>Estruturação, reforma e ampliação da Fundação Ezequiel Dias – Funed</t>
+  </si>
+  <si>
+    <t>Estudo de viabilidade técnica e financeira e modelo de gestão da reestruturação da Fundação Ezequiel Dias – Funed</t>
+  </si>
+  <si>
+    <t>Convivência com a Seca - Construção de cisternas</t>
+  </si>
+  <si>
+    <t>Georreferenciamento de bens culturais protegidos</t>
+  </si>
+  <si>
+    <t>Fortalecimento da estrutura e dos processos do Instituto Mineiro de Agropecuária</t>
+  </si>
+  <si>
+    <t>Implantação do Sistema de Gestão de Processos (BPMS) no Instituto Mineiro de Agropecuária (IMA)</t>
+  </si>
+  <si>
+    <t>Reestruturação do laboratório de química agropecuária do Instituto Mineiro de Agropecuária</t>
+  </si>
+  <si>
+    <t>Revitalização do Parque de Exposições Bolivar de Andrade</t>
+  </si>
+  <si>
+    <t>Implantação da Ouvidoria 4.0 e Ouvidoria Móvel</t>
+  </si>
+  <si>
+    <t>Construção do Núcleo Integrado de Perícias da Polícia Civil de Minas Gerais</t>
+  </si>
+  <si>
+    <t>Estruturação operacional da Polícia Civil de Minas Gerais</t>
+  </si>
+  <si>
+    <t>Projeto ABIS - Sistema Automatizado de Identificação Biométrica</t>
+  </si>
+  <si>
+    <t>Ampliação da rede de rádio digital no interior do Estado de Minas Gerais</t>
+  </si>
+  <si>
+    <t>Fortalecimento do atendimento à saúde militar</t>
+  </si>
+  <si>
+    <t>Proteção policial individual e do cidadão mineiro</t>
+  </si>
+  <si>
+    <t>Segurança Rural e de Áreas de Risco</t>
+  </si>
+  <si>
+    <t>Plano de Desenvolvimento da Cadeia Agropecuária</t>
+  </si>
+  <si>
+    <t>Fortalecimento da competitividade turística de Minas Gerais</t>
+  </si>
+  <si>
+    <t>Pesquisas, Tendências e Monitoramento da Cultura e do Turismo</t>
+  </si>
+  <si>
+    <t>Plano de Desenvolvimento Integrado do Turismo em Minas Gerais</t>
+  </si>
+  <si>
+    <t>Elaboração de instrumentos de gestão para desenvolvimento de mineração sustentável e competitiva - Avaliação Ambiental Estratégica</t>
+  </si>
+  <si>
+    <t>Elaboração de instrumentos de gestão para desenvolvimento de mineração sustentável e competitiva - Elaboração do Plano Estadual da Mineração de Minas Gerais</t>
+  </si>
+  <si>
+    <t>Melhoria da infraestrutura dos municípios</t>
+  </si>
+  <si>
+    <t>Melhoria da infraestrutura dos municípios - Outros repasses</t>
+  </si>
+  <si>
+    <t>Recuperação de rodovias pavimentadas em pior estado, conforme avaliação técnica do DER-MG / conclusão de corredor logístico estruturante, conforme critérios técnicos da Seinfra / melhoria da infraestrutura dos municípios</t>
+  </si>
+  <si>
+    <t>Prevenção de Enchentes - Construção de Bacias de Contenção no Córrego Ferrugem</t>
+  </si>
+  <si>
+    <t>Prevenção de Enchentes - Desapropriação para construção de bacias de contenção no Córrego Riacho das Pedras.</t>
+  </si>
+  <si>
+    <t>Implantação do Rodoanel da Região Metropolitana de Belo Horizonte</t>
+  </si>
+  <si>
+    <t>Realização de obras rodoviárias - Caeté - Barão de Cocais e Contorno de Barão de Cocais</t>
+  </si>
+  <si>
+    <t>Recuperação de rodovias pavimentadas em pior estado, conforme avaliação técnica do DER-MG/conclusão de corredor logístico estruturante, conforme critérios técnicos da SEINFRA</t>
+  </si>
+  <si>
+    <t>Construção de pontes em São Francisco, Manga e São Romão sobre o Rio São Francisco</t>
+  </si>
+  <si>
+    <t>Reintegração social e humanização do sistema prisional</t>
+  </si>
+  <si>
+    <t>Contratações temporárias</t>
+  </si>
+  <si>
+    <t>Estruturas de apoio</t>
+  </si>
+  <si>
+    <t>Melhoria da estrutura logística e energética da Cidade Administrativa para redução de custos</t>
+  </si>
+  <si>
+    <t>Ressarcimentos de despesas públicas</t>
+  </si>
+  <si>
+    <t>Ampliação de postos de abastecimento próprios do Estado</t>
+  </si>
+  <si>
+    <t>Conclusão de obra e Equipagem de Hospitais Regionais</t>
+  </si>
+  <si>
     <t>Ações de Prevenção e Combate a Incêndio em Unidades de Conservação Estaduais</t>
   </si>
   <si>
-    <t>Secretaria de Estado de Meio Ambiente e Desenvolvimento Sustentável</t>
+    <t>Consolidação das unidades de conservação no Estado de Minas Gerais</t>
+  </si>
+  <si>
+    <t>Construção e/ou manutenção de Centros de Triagem e Reabilitação de Animais Silvestres no Estado de Minas Gerais</t>
+  </si>
+  <si>
+    <t>Consultoria técnica sobre a descaracterização das barragens I e II da Mundo Mineração Ltda.</t>
+  </si>
+  <si>
+    <t>Fortalecimento da estrutura de fiscalização do Sistema Estadual de Meio Ambiente</t>
+  </si>
+  <si>
+    <t>Implantação de Fábrica de Software para construção de sistema de governança ambiental</t>
+  </si>
+  <si>
+    <t>Ressarcimentos e contratações temporárias</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* \-??_-;_-@_-"/>
+    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
-      <color rgb="FF000000"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <charset val="1"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF000000"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <charset val="1"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -109,16 +267,25 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -434,60 +601,788 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D55"/>
   <sheetFormatPr defaultColWidth="28.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.28515625" customWidth="1"/>
-    <col min="2" max="2" width="6.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20" customWidth="1"/>
-    <col min="4" max="4" width="15.140625" customWidth="1"/>
-    <col min="5" max="5" width="28.85546875" customWidth="1"/>
-    <col min="6" max="6" width="28.7109375" style="1"/>
+    <col min="2" max="2" width="42.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.85546875" customWidth="1"/>
+    <col min="4" max="4" width="28.7109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="3" t="s">
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="5">
+        <v>9288176</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D2" s="6">
+        <v>23131467.960000001</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="5">
+        <v>9288139</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D3" s="6">
+        <v>3200000</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" s="5">
+        <v>9288185</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D4" s="6">
+        <v>2000000</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" s="5">
+        <v>9288135</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D5" s="1">
+        <v>1345000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" s="5">
+        <v>9288169</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D6" s="1">
+        <v>33248482</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" s="5">
+        <v>9288168</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D7" s="1">
+        <v>130000000</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" s="5">
+        <v>9288167</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D8" s="1">
+        <v>3773400</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" s="5">
+        <v>9288155</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D9" s="1">
+        <v>5100000</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" s="5">
+        <v>9288212</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C10" s="4" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2">
+      <c r="D10" s="1">
+        <v>2050000000</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" s="5">
+        <v>9288136</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D11" s="1">
+        <v>111480000</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" s="5">
+        <v>9288214</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D12" s="1">
+        <v>199489167.000002</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" s="5">
+        <v>9288209</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D13" s="1">
+        <v>1200000</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" s="5">
+        <v>9288147</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D14" s="1">
+        <v>14817323</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" s="5">
+        <v>9288141</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D15" s="1">
+        <v>500000</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" s="5">
+        <v>9288142</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D16" s="1">
+        <v>29712000</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" s="5">
+        <v>9288193</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D17" s="1">
+        <v>3900000</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" s="5">
+        <v>9288194</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D18" s="1">
+        <v>3600000</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" s="5">
+        <v>9288149</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D19" s="1">
+        <v>5000000</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" s="5">
+        <v>9288143</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D20" s="1">
+        <v>728000</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" s="5">
+        <v>9288144</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D21" s="1">
+        <v>49000000</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22" s="5">
+        <v>9288196</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D22" s="1">
+        <v>1800000</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23" s="5">
+        <v>9288145</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D23" s="1">
+        <v>94500000</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24" s="5">
+        <v>9288137</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D24" s="1">
+        <v>100000000</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A25" s="5">
+        <v>9288148</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D25" s="1">
+        <v>114995000</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26" s="5">
+        <v>9288138</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D26" s="1">
+        <v>17996000</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A27" s="5">
+        <v>9288150</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D27" s="1">
+        <v>10671300</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A28" s="5">
+        <v>9321270</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D28" s="1">
+        <v>800000</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A29" s="5">
+        <v>9288152</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D29" s="1">
+        <v>15130000</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A30" s="5">
+        <v>9288153</v>
+      </c>
+      <c r="B30" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D30" s="1">
+        <v>3000000</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A31" s="5">
+        <v>9288154</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D31" s="1">
+        <v>650000</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A32" s="5">
+        <v>9288210</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D32" s="1">
+        <v>2500000</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A33" s="5">
+        <v>9288211</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D33" s="1">
+        <v>3200000</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A34" s="5">
+        <v>9288130</v>
+      </c>
+      <c r="B34" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D34" s="1">
+        <v>1107550000</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A35" s="5">
+        <v>9288177</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D35" s="1">
+        <v>100370000</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A36" s="5">
+        <v>9288130</v>
+      </c>
+      <c r="B36" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="C36" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D36" s="1">
+        <v>450000000</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A37" s="5">
+        <v>9288178</v>
+      </c>
+      <c r="B37" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="C37" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D37" s="1">
+        <v>253000000</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A38" s="5">
+        <v>9288179</v>
+      </c>
+      <c r="B38" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="C38" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D38" s="1">
+        <v>45000000</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A39" s="5">
+        <v>9288180</v>
+      </c>
+      <c r="B39" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="C39" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D39" s="1">
+        <v>3072030000</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A40" s="5">
+        <v>9288134</v>
+      </c>
+      <c r="B40" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C40" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D40" s="1">
+        <v>98860000</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A41" s="5">
+        <v>9288133</v>
+      </c>
+      <c r="B41" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="C41" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D41" s="1">
+        <v>700000000</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A42" s="5">
+        <v>9288132</v>
+      </c>
+      <c r="B42" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="C42" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D42" s="1">
+        <v>300000000</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A43" s="5">
+        <v>9288181</v>
+      </c>
+      <c r="B43" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="C43" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D43" s="1">
+        <v>552000</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A44" s="5">
+        <v>9288192</v>
+      </c>
+      <c r="B44" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="C44" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="D44" s="1">
+        <v>100000000</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A45" s="5">
+        <v>9288190</v>
+      </c>
+      <c r="B45" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="C45" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="D45" s="1">
+        <v>99720000</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A46" s="5">
+        <v>9288183</v>
+      </c>
+      <c r="B46" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="C46" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D46" s="1">
+        <v>8000000</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A47" s="5">
+        <v>9288191</v>
+      </c>
+      <c r="B47" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C47" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="D47" s="1">
+        <v>210000000</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A48" s="5">
+        <v>9288182</v>
+      </c>
+      <c r="B48" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="C48" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D48" s="1">
+        <v>7000000</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A49" s="5">
+        <v>9288198</v>
+      </c>
+      <c r="B49" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="C49" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D49" s="1">
+        <v>985935044</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A50" s="5">
         <v>9288186</v>
       </c>
-      <c r="B2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C2">
-        <v>1371</v>
-      </c>
-      <c r="D2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E2" t="s">
-        <v>7</v>
-      </c>
-      <c r="F2" s="1">
+      <c r="B50" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="C50" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D50" s="1">
         <v>3000000</v>
       </c>
     </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A51" s="5">
+        <v>9288187</v>
+      </c>
+      <c r="B51" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="C51" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D51" s="1">
+        <v>36000000</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A52" s="5">
+        <v>9288188</v>
+      </c>
+      <c r="B52" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="C52" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D52" s="1">
+        <v>8647600</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A53" s="5">
+        <v>9288189</v>
+      </c>
+      <c r="B53" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="C53" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D53" s="1">
+        <v>300000</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A54" s="5">
+        <v>9288195</v>
+      </c>
+      <c r="B54" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="C54" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D54" s="1">
+        <v>749679</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A55" s="5">
+        <v>9288213</v>
+      </c>
+      <c r="B55" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="C55" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D55" s="1">
+        <v>23000005</v>
+      </c>
+    </row>
   </sheetData>
-  <pageMargins left="0.51180555555555496" right="0.51180555555555496" top="0.78749999999999998" bottom="0.78749999999999998" header="0.51180555555555496" footer="0.51180555555555496"/>
-  <pageSetup paperSize="9" firstPageNumber="0" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Testa validação de arquivo
</commit_message>
<xml_diff>
--- a/data/raw/projetos_acordo_judicial_reparacao_vale.xlsx
+++ b/data/raw/projetos_acordo_judicial_reparacao_vale.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hugos\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\m13368964\Documents\Documents\1.CGE\tele-trabalho\GIT\transparencia-mg\acordo-judicial-vale\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="63">
   <si>
     <t>projeto</t>
   </si>
@@ -223,6 +223,9 @@
   </si>
   <si>
     <t>Ressarcimentos e contratações temporárias</t>
+  </si>
+  <si>
+    <t>z.Ressarcimentos e contratações temporárias</t>
   </si>
 </sst>
 </file>
@@ -1221,7 +1224,7 @@
         <v>49</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D44" s="1">
         <v>100000000</v>

</xml_diff>

<commit_message>
Corrige erro no arquivo
</commit_message>
<xml_diff>
--- a/data/raw/projetos_acordo_judicial_reparacao_vale.xlsx
+++ b/data/raw/projetos_acordo_judicial_reparacao_vale.xlsx
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="62">
   <si>
     <t>projeto</t>
   </si>
@@ -223,9 +223,6 @@
   </si>
   <si>
     <t>Ressarcimentos e contratações temporárias</t>
-  </si>
-  <si>
-    <t>z.Ressarcimentos e contratações temporárias</t>
   </si>
 </sst>
 </file>
@@ -1224,7 +1221,7 @@
         <v>49</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D44" s="1">
         <v>100000000</v>

</xml_diff>